<commit_message>
corretced the SL order logic
</commit_message>
<xml_diff>
--- a/pnl_tracker.xlsx
+++ b/pnl_tracker.xlsx
@@ -412,16 +412,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="3"/>
+    <col width="23" customWidth="1" min="2" max="3"/>
     <col width="5" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="7"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,6 +605,30 @@
         <v>-28.2</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-02-11 10.18.37</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY2621726000PE</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>65</v>
+      </c>
+      <c r="D8" t="n">
+        <v>114.65</v>
+      </c>
+      <c r="E8" t="n">
+        <v>134.7</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1517.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>